<commit_message>
Update dual concert ticketing system
</commit_message>
<xml_diff>
--- a/data/seat_map_tp.xlsx
+++ b/data/seat_map_tp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bryanwl/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bryanwl/Documents/ntuco2026tp/ntuco2026tp/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5783E15-0973-6F46-BE83-9E768607D82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BD841AF-A2C5-0243-8903-168CF0CA27FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4920,7 +4920,7 @@
         <v>19</v>
       </c>
       <c r="AZ28" s="7">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="BA28" s="6"/>
       <c r="BB28" s="7"/>

</xml_diff>